<commit_message>
#1 Updated with issues resolved
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Issue#2/Boost_Regulator.xlsx
+++ b/Documents/Dev-Files/Issue#2/Boost_Regulator.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$L$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$M$16</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="29">
   <si>
     <t>Output Type</t>
   </si>
@@ -56,15 +56,6 @@
     <t>10000+</t>
   </si>
   <si>
-    <t>TPS61322</t>
-  </si>
-  <si>
-    <t>MAX858CSA+T</t>
-  </si>
-  <si>
-    <t>2.7-6</t>
-  </si>
-  <si>
     <t>Iout(mA)</t>
   </si>
   <si>
@@ -98,9 +89,6 @@
     <t>TPS61023DRLR</t>
   </si>
   <si>
-    <t>https://www.lcsc.com/product-detail/DC-DC-Converters_Texas-Instruments-TPS61023DRLR_C919459.html</t>
-  </si>
-  <si>
     <t>Links</t>
   </si>
   <si>
@@ -110,20 +98,29 @@
     <t>Preferred</t>
   </si>
   <si>
-    <t>https://www.mvele.ca/Showpro.html?search1=TPS61322DBZR</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
     <t>BOOST REGULATOR</t>
+  </si>
+  <si>
+    <t>LCSC</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>Datasheet</t>
+  </si>
+  <si>
+    <t>TPS613222ADBVR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,14 +155,6 @@
       <color rgb="FF24292F"/>
       <name val="Segoe UI"/>
       <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="14"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -204,7 +193,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -487,6 +476,80 @@
         <color indexed="64"/>
       </right>
       <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -497,7 +560,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -514,50 +577,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -565,45 +592,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -612,6 +600,99 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -893,91 +974,94 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="50.5703125" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="1" max="1" width="37.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="15.28515625" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" customWidth="1"/>
-    <col min="9" max="9" width="22.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="17.42578125" customWidth="1"/>
+    <col min="9" max="9" width="21.7109375" customWidth="1"/>
     <col min="10" max="10" width="22.85546875" customWidth="1"/>
-    <col min="11" max="11" width="60.5703125" customWidth="1"/>
-    <col min="12" max="12" width="23.42578125" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="19.5703125" customWidth="1"/>
+    <col min="13" max="13" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="C2" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="27"/>
-    </row>
-    <row r="3" spans="1:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="28"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="30"/>
-    </row>
-    <row r="4" spans="1:12" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="10"/>
-    </row>
-    <row r="6" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="13"/>
-    </row>
-    <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C2" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="23"/>
+    </row>
+    <row r="3" spans="1:13" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="24"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="26"/>
+    </row>
+    <row r="4" spans="1:13" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="34"/>
+      <c r="J5" s="34"/>
+      <c r="K5" s="34"/>
+      <c r="L5" s="35"/>
+      <c r="M5" s="36"/>
+    </row>
+    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="37"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
+      <c r="J6" s="38"/>
+      <c r="K6" s="38"/>
+      <c r="L6" s="39"/>
+      <c r="M6" s="40"/>
+    </row>
+    <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>0</v>
@@ -991,14 +1075,15 @@
       <c r="J7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="K7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="L7" s="35" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K7" s="41" t="s">
+        <v>23</v>
+      </c>
+      <c r="L7" s="18"/>
+      <c r="M7" s="43" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6"/>
       <c r="B8" s="7">
         <v>1.8</v>
@@ -1016,21 +1101,22 @@
         <v>100</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>7</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="J8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K8" s="36"/>
-      <c r="L8" s="37"/>
-    </row>
-    <row r="9" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K8" s="42"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="44"/>
+    </row>
+    <row r="9" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1043,8 +1129,9 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
-    </row>
-    <row r="10" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M9" s="2"/>
+    </row>
+    <row r="10" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1057,55 +1144,58 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="1:12" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="16"/>
-    </row>
-    <row r="12" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="31"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="32"/>
-      <c r="L12" s="33"/>
-    </row>
-    <row r="13" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M10" s="2"/>
+    </row>
+    <row r="11" spans="1:13" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="28"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="29"/>
+    </row>
+    <row r="12" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="30"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="32"/>
+    </row>
+    <row r="13" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>0</v>
@@ -1120,13 +1210,16 @@
         <v>3</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="L13" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="L13" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1138,242 +1231,236 @@
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
       <c r="K14" s="4"/>
-      <c r="L14" s="5"/>
-    </row>
-    <row r="15" spans="1:12" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" s="18">
+      <c r="L14" s="20"/>
+      <c r="M14" s="5"/>
+    </row>
+    <row r="15" spans="1:13" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="9">
         <v>0.9</v>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="9">
         <v>5.5</v>
       </c>
-      <c r="D15" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="E15" s="18">
+      <c r="D15" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="9">
         <v>900</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="9">
         <v>6.5</v>
       </c>
-      <c r="G15" s="18" t="s">
+      <c r="G15" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H15" s="18" t="s">
+      <c r="H15" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I15" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="J15" s="18" t="s">
+      <c r="I15" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J15" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K15" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="L15" s="20" t="s">
+      <c r="K15" s="17" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" ht="56.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="17" t="s">
+      <c r="L15" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="M15" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="18">
+    </row>
+    <row r="16" spans="1:13" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="7">
         <v>0.5</v>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="7">
         <v>5.5</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="7">
         <v>1800</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="7">
         <v>20</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="G16" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H16" s="18" t="s">
+      <c r="H16" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I16" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" s="18" t="s">
+      <c r="I16" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="J16" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="K16" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="L16" s="22"/>
-    </row>
-    <row r="17" spans="1:14" ht="62.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="7">
-        <v>0.8</v>
-      </c>
-      <c r="C17" s="7">
-        <v>6</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" s="7">
-        <v>60</v>
-      </c>
-      <c r="F17" s="7">
+      <c r="K16" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="G17" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="K17" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="L17" s="24"/>
-    </row>
-    <row r="18" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A18" s="38"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="38"/>
-      <c r="J18" s="38"/>
-      <c r="K18" s="38"/>
-      <c r="L18" s="39"/>
-      <c r="M18" s="40"/>
-      <c r="N18" s="40"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="40"/>
-      <c r="B19" s="40"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="40"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="40"/>
-      <c r="J19" s="40"/>
-      <c r="K19" s="40"/>
-      <c r="L19" s="40"/>
-      <c r="M19" s="40"/>
-      <c r="N19" s="40"/>
-    </row>
-    <row r="20" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A20" s="41"/>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="40"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="40"/>
-      <c r="J20" s="40"/>
-      <c r="K20" s="40"/>
-      <c r="L20" s="40"/>
-      <c r="M20" s="40"/>
-      <c r="N20" s="40"/>
-    </row>
-    <row r="21" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A21" s="41"/>
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="40"/>
-      <c r="J21" s="40"/>
-      <c r="K21" s="40"/>
-      <c r="L21" s="40"/>
-      <c r="M21" s="40"/>
-      <c r="N21" s="40"/>
-    </row>
-    <row r="22" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A22" s="41"/>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="40"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="40"/>
-      <c r="I22" s="40"/>
-      <c r="J22" s="40"/>
-      <c r="K22" s="40"/>
-      <c r="L22" s="40"/>
-      <c r="M22" s="40"/>
-      <c r="N22" s="40"/>
-    </row>
-    <row r="23" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A23" s="41"/>
-      <c r="B23" s="40"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="40"/>
-      <c r="J23" s="40"/>
-      <c r="K23" s="40"/>
-      <c r="L23" s="40"/>
-      <c r="M23" s="40"/>
-      <c r="N23" s="40"/>
-    </row>
-    <row r="24" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="L16" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="M16" s="12"/>
+    </row>
+    <row r="17" spans="1:15" ht="62.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15"/>
+      <c r="M17" s="14"/>
+    </row>
+    <row r="18" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="15"/>
+      <c r="O18" s="15"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="15"/>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
+      <c r="O19" s="15"/>
+    </row>
+    <row r="20" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A20" s="16"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+    </row>
+    <row r="21" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A21" s="16"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
+      <c r="L21" s="15"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15"/>
+      <c r="O21" s="15"/>
+    </row>
+    <row r="22" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A22" s="16"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15"/>
+      <c r="L22" s="15"/>
+      <c r="M22" s="15"/>
+      <c r="N22" s="15"/>
+      <c r="O22" s="15"/>
+    </row>
+    <row r="23" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A23" s="16"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="15"/>
+      <c r="L23" s="15"/>
+      <c r="M23" s="15"/>
+      <c r="N23" s="15"/>
+      <c r="O23" s="15"/>
+    </row>
+    <row r="24" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
     </row>
-    <row r="25" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
     </row>
-    <row r="26" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:14" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="C2:I3"/>
-    <mergeCell ref="A11:L12"/>
-    <mergeCell ref="A5:L6"/>
+    <mergeCell ref="A11:M12"/>
+    <mergeCell ref="A5:M6"/>
     <mergeCell ref="K7:K8"/>
-    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="M7:M8"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="K16" r:id="rId1"/>
     <hyperlink ref="K15" r:id="rId2"/>
+    <hyperlink ref="L15" r:id="rId3"/>
+    <hyperlink ref="L16" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="29" orientation="portrait" r:id="rId3"/>
+  <pageSetup scale="29" orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#2 File Updated with proper description
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Issue#2/Boost_Regulator.xlsx
+++ b/Documents/Dev-Files/Issue#2/Boost_Regulator.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="47">
   <si>
     <t>Output Type</t>
   </si>
@@ -149,32 +149,32 @@
     <t>1.23-34</t>
   </si>
   <si>
-    <t>Complex Application Circuit</t>
-  </si>
-  <si>
-    <t>Expensive</t>
-  </si>
-  <si>
     <t>TPS613222ADBVT</t>
   </si>
   <si>
-    <t>Second Preference</t>
-  </si>
-  <si>
     <t>Cost($)</t>
   </si>
   <si>
-    <t>Preferred because of 
-1.Most Cheap
-2.Simple Application Circuit
-3.High switching Frequency</t>
+    <t>It is designed for high power system with long range input with fewer external components. It is also cheap hence it is on Second Preference.</t>
+  </si>
+  <si>
+    <t>This IC is of high Efficiency with short circuit protection. It is equipped with simple application circuit, but is not preferred because of high cost.</t>
+  </si>
+  <si>
+    <t>This IC is Synchronous with high efficiency and simple circuitry. It includes Over Current and Over Voltage Protection, but it is not preferred because it is expensive.</t>
+  </si>
+  <si>
+    <t>This IC is of high efficiency with Synchronous configuration and fewer external components but its cost is greater than the above two, hence less preferred.</t>
+  </si>
+  <si>
+    <t>This IC is preferred because of lowest cost and it has simple application circuit with less external components and high efficiency.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -232,25 +232,8 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -281,8 +264,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="28">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -438,21 +427,6 @@
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -631,12 +605,66 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -649,16 +677,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -666,117 +691,141 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1075,72 +1124,72 @@
     <col min="11" max="12" width="22.85546875" customWidth="1"/>
     <col min="13" max="13" width="15" customWidth="1"/>
     <col min="14" max="14" width="19.5703125" customWidth="1"/>
-    <col min="15" max="15" width="35.85546875" customWidth="1"/>
+    <col min="15" max="15" width="68.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D2" s="13" t="s">
+    <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D2" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="15"/>
-    </row>
-    <row r="3" spans="1:15" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="16"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="18"/>
-    </row>
-    <row r="4" spans="1:15" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="34"/>
+    </row>
+    <row r="3" spans="1:17" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D3" s="35"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="37"/>
+    </row>
+    <row r="4" spans="1:17" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="28"/>
-    </row>
-    <row r="6" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="29"/>
-      <c r="B6" s="38"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
-      <c r="K6" s="30"/>
-      <c r="L6" s="30"/>
-      <c r="M6" s="30"/>
-      <c r="N6" s="31"/>
-      <c r="O6" s="32"/>
-    </row>
-    <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="35" t="s">
+      <c r="B5" s="45"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="46"/>
+      <c r="I5" s="46"/>
+      <c r="J5" s="46"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="46"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="47"/>
+      <c r="O5" s="48"/>
+    </row>
+    <row r="6" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="49"/>
+      <c r="B6" s="50"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
+      <c r="I6" s="51"/>
+      <c r="J6" s="51"/>
+      <c r="K6" s="51"/>
+      <c r="L6" s="51"/>
+      <c r="M6" s="51"/>
+      <c r="N6" s="52"/>
+      <c r="O6" s="53"/>
+    </row>
+    <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="56" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -1170,22 +1219,22 @@
       <c r="K7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="L7" s="35" t="s">
+      <c r="L7" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="33" t="s">
+      <c r="M7" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="N7" s="35" t="s">
+      <c r="N7" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="O7" s="35" t="s">
+      <c r="O7" s="56" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="36"/>
-      <c r="B8" s="36"/>
+    <row r="8" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="57"/>
+      <c r="B8" s="57"/>
       <c r="C8" s="6">
         <v>1.8</v>
       </c>
@@ -1213,12 +1262,12 @@
       <c r="K8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="L8" s="36"/>
-      <c r="M8" s="34"/>
-      <c r="N8" s="36"/>
-      <c r="O8" s="36"/>
-    </row>
-    <row r="9" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L8" s="57"/>
+      <c r="M8" s="55"/>
+      <c r="N8" s="57"/>
+      <c r="O8" s="57"/>
+    </row>
+    <row r="9" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1235,7 +1284,7 @@
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1252,47 +1301,47 @@
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="1:15" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+    <row r="11" spans="1:17" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20"/>
-      <c r="M11" s="20"/>
-      <c r="N11" s="20"/>
-      <c r="O11" s="21"/>
-    </row>
-    <row r="12" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="22"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
-      <c r="J12" s="23"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="23"/>
-      <c r="M12" s="23"/>
-      <c r="N12" s="23"/>
-      <c r="O12" s="24"/>
-    </row>
-    <row r="13" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="39"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="39"/>
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
+      <c r="L11" s="39"/>
+      <c r="M11" s="39"/>
+      <c r="N11" s="39"/>
+      <c r="O11" s="40"/>
+    </row>
+    <row r="12" spans="1:17" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="41"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="42"/>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
+      <c r="K12" s="42"/>
+      <c r="L12" s="42"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="42"/>
+      <c r="O12" s="43"/>
+    </row>
+    <row r="13" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="12" t="s">
         <v>31</v>
       </c>
       <c r="C13" s="4" t="s">
@@ -1323,7 +1372,7 @@
         <v>3</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="M13" s="4" t="s">
         <v>20</v>
@@ -1335,7 +1384,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1352,168 +1401,170 @@
       <c r="N14" s="4"/>
       <c r="O14" s="5"/>
     </row>
-    <row r="15" spans="1:15" ht="87.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="47" t="s">
+    <row r="15" spans="1:17" ht="87.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="48">
+      <c r="C15" s="17">
         <v>0.5</v>
       </c>
-      <c r="D15" s="48">
+      <c r="D15" s="17">
         <v>5.5</v>
       </c>
-      <c r="E15" s="48" t="s">
+      <c r="E15" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="F15" s="48">
+      <c r="F15" s="17">
         <v>1800</v>
       </c>
-      <c r="G15" s="48">
+      <c r="G15" s="17">
         <v>20</v>
       </c>
-      <c r="H15" s="48" t="s">
+      <c r="H15" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="I15" s="48" t="s">
+      <c r="I15" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="J15" s="48" t="s">
+      <c r="J15" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="K15" s="48" t="s">
+      <c r="K15" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="L15" s="48">
+      <c r="L15" s="17">
         <v>0.33</v>
       </c>
-      <c r="M15" s="49" t="s">
+      <c r="M15" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="N15" s="49" t="s">
+      <c r="N15" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="O15" s="50" t="s">
+      <c r="O15" s="19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="24">
+        <v>1.2</v>
+      </c>
+      <c r="D16" s="24">
+        <v>12</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="F16" s="24">
+        <v>350</v>
+      </c>
+      <c r="G16" s="24">
+        <v>1</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="I16" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="J16" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="L16" s="24">
+        <v>0.76</v>
+      </c>
+      <c r="M16" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="N16" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="O16" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="9"/>
+    </row>
+    <row r="17" spans="1:17" ht="66" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="21">
+        <v>0.9</v>
+      </c>
+      <c r="D17" s="21">
+        <v>5.5</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="21">
+        <v>900</v>
+      </c>
+      <c r="G17" s="21">
+        <v>6.5</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I17" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="J17" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="K17" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="L17" s="21">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="M17" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="N17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="O17" s="23" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="8">
-        <v>0.9</v>
-      </c>
-      <c r="D16" s="8">
-        <v>5.5</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="8">
-        <v>900</v>
-      </c>
-      <c r="G16" s="8">
-        <v>6.5</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J16" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="K16" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L16" s="8">
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="M16" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="N16" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="O16" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+    <row r="18" spans="1:17" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B18" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C18" s="8">
         <v>0.6</v>
-      </c>
-      <c r="D17" s="8">
-        <v>5.5</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="F17" s="8">
-        <v>800</v>
-      </c>
-      <c r="G17" s="8">
-        <v>11</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="K17" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L17" s="8">
-        <v>2.88</v>
-      </c>
-      <c r="M17" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="N17" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="O17" s="43" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" s="8">
-        <v>0.9</v>
       </c>
       <c r="D18" s="8">
         <v>5.5</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="F18" s="8">
-        <v>850</v>
+        <v>800</v>
       </c>
       <c r="G18" s="8">
-        <v>1.2E-2</v>
+        <v>11</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>6</v>
@@ -1528,41 +1579,39 @@
         <v>8</v>
       </c>
       <c r="L18" s="8">
-        <v>2.82</v>
-      </c>
-      <c r="M18" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="N18" s="12" t="s">
+        <v>2.88</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="N18" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="O18" s="14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="79.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="O18" s="43" t="s">
-        <v>41</v>
-      </c>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="10"/>
-    </row>
-    <row r="19" spans="1:17" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="41" t="s">
-        <v>36</v>
-      </c>
       <c r="B19" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C19" s="6">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="D19" s="6">
-        <v>12</v>
+        <v>5.5</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F19" s="6">
-        <v>350</v>
+        <v>850</v>
       </c>
       <c r="G19" s="6">
-        <v>1</v>
+        <v>1.2E-2</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>6</v>
@@ -1577,76 +1626,76 @@
         <v>8</v>
       </c>
       <c r="L19" s="6">
-        <v>0.76</v>
-      </c>
-      <c r="M19" s="42" t="s">
+        <v>2.82</v>
+      </c>
+      <c r="M19" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="N19" s="42" t="s">
-        <v>36</v>
-      </c>
-      <c r="O19" s="44" t="s">
-        <v>40</v>
-      </c>
-      <c r="P19" s="46"/>
-      <c r="Q19" s="10"/>
+      <c r="N19" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="O19" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="P19" s="9"/>
+      <c r="Q19" s="9"/>
     </row>
     <row r="20" spans="1:17" ht="87" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="40"/>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10"/>
-      <c r="O20" s="10"/>
-      <c r="P20" s="10"/>
-      <c r="Q20" s="45"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="9"/>
+      <c r="P20" s="9"/>
+      <c r="Q20" s="15"/>
     </row>
     <row r="21" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="10"/>
-      <c r="Q21" s="10"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
     </row>
     <row r="22" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10"/>
-      <c r="O22" s="10"/>
-      <c r="P22" s="10"/>
-      <c r="Q22" s="10"/>
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="9"/>
+      <c r="Q22" s="9"/>
     </row>
     <row r="23" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
@@ -1670,29 +1719,29 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="A7:A8"/>
     <mergeCell ref="D2:J3"/>
     <mergeCell ref="A11:O12"/>
     <mergeCell ref="A5:O6"/>
     <mergeCell ref="M7:M8"/>
     <mergeCell ref="O7:O8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="A7:A8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="N16" r:id="rId1"/>
-    <hyperlink ref="M17" r:id="rId2"/>
-    <hyperlink ref="N17" r:id="rId3"/>
-    <hyperlink ref="N18" r:id="rId4"/>
-    <hyperlink ref="M18" r:id="rId5"/>
-    <hyperlink ref="M19" r:id="rId6"/>
-    <hyperlink ref="N19" r:id="rId7"/>
+    <hyperlink ref="N17" r:id="rId1"/>
+    <hyperlink ref="M18" r:id="rId2"/>
+    <hyperlink ref="N18" r:id="rId3"/>
+    <hyperlink ref="N19" r:id="rId4"/>
+    <hyperlink ref="M19" r:id="rId5"/>
+    <hyperlink ref="M16" r:id="rId6"/>
+    <hyperlink ref="N16" r:id="rId7"/>
     <hyperlink ref="N15" r:id="rId8"/>
     <hyperlink ref="M15" r:id="rId9"/>
-    <hyperlink ref="M16" r:id="rId10"/>
+    <hyperlink ref="M17" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="28" orientation="portrait" r:id="rId11"/>
+  <pageSetup scale="26" orientation="portrait" r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>